<commit_message>
site build 2026-10-08 21:25
</commit_message>
<xml_diff>
--- a/models/sovereigns/Kenya_Sovereign_Model.xlsx
+++ b/models/sovereigns/Kenya_Sovereign_Model.xlsx
@@ -647,12 +647,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>07-Oct-26</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Central Bank of Kenya MPC communiqué (Central Bank Rate)</t>
+          <t>CBK MPC</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>6.8</v>
+        <v>6.76</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -700,12 +700,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Kenya National Bureau of Statistics</t>
+          <t>IMF data portal; KNBS (6.8%)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>30-Sep-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -736,14 +736,10 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -783,7 +779,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>National Treasury and Economic Planning</t>
+          <t>National Treasury</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -793,7 +789,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Total public debt Ksh 13.01 trillion, end-June 2026; statutory anchor 55% of GDP</t>
+          <t>public debt Ksh 13.01tn; 55% debt anchor</t>
         </is>
       </c>
     </row>
@@ -830,12 +826,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FY2025/26 (projected, Ksh 1.199 trillion deficit)</t>
+          <t>FY2025/26 (projected, Ksh 1.199tn deficit; audited outturn not in hand)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>National Treasury and Economic Planning</t>
+          <t>National Treasury</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -878,7 +874,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FY2025/26 (approx., share of ordinary revenue)</t>
+          <t>approximate, ordinary revenue, latest</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -888,7 +884,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Jun-26</t>
+          <t>Jul-26</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -936,14 +932,10 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -971,14 +963,10 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -996,12 +984,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>07-Oct-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Central Bank of Kenya</t>
+          <t>CBK</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1011,7 +999,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>CBK gross FX reserves (gold treatment not stated)</t>
+          <t>gross, CBK headline; composition and encumbrances not stated (IMF series shows gold negligible)</t>
         </is>
       </c>
     </row>
@@ -1058,14 +1046,10 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1144,14 +1128,10 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1313,6 +1293,11 @@
       <c r="A33" t="inlineStr">
         <is>
           <t>IMF</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>None; prior EFF/ECF/RSF expired uncompleted Apr-25, successor talks ongoing</t>
         </is>
       </c>
     </row>
@@ -1361,9 +1346,15 @@
           <t>nominal_gdp_usd_bn</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
+      <c r="B2" s="2" t="n">
+        <v>147.265</v>
+      </c>
       <c r="C2" s="2" t="n"/>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>IMF WEO 2026E, Sep-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1371,9 +1362,15 @@
           <t>real_gdp_growth_pct</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
+      <c r="B3" s="2" t="n">
+        <v>4.5</v>
+      </c>
       <c r="C3" s="2" t="n"/>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>IMF WEO 2026E, Sep-26</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1391,9 +1388,15 @@
           <t>current_account_pct_gdp</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n"/>
+      <c r="B5" s="2" t="n">
+        <v>-4.1</v>
+      </c>
       <c r="C5" s="2" t="n"/>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>IMF WEO 2026E, Sep-26</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">

</xml_diff>

<commit_message>
site build 2026-10-15 12:04
</commit_message>
<xml_diff>
--- a/models/sovereigns/Kenya_Sovereign_Model.xlsx
+++ b/models/sovereigns/Kenya_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 09-Oct-26</t>
+          <t>as of 15-Oct-26</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 12-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/kenya.json</t>
+          <t>built 15-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/kenya.json</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Central Bank of Kenya, MPC (CBR held)</t>
+          <t>CBK MPC press release</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -700,12 +700,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>IMF data portal; KNBS (6.8%)</t>
+          <t>KNBS / IMF data portal</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>07-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -784,12 +784,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>Jun-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>public debt Ksh 13.01tn; 55% debt anchor</t>
+          <t>Public debt Ksh13.01tn; National Treasury anchor 55% of GDP</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FY2025/26 (projected; audited outturn not in hand)</t>
+          <t>FY2025/26 (projection, Ksh1.199tn deficit)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Jul-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -872,15 +872,19 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>FY2025/26 (approximate, ordinary revenue)</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>National Treasury / World Bank (approximate, share of ordinary revenue)</t>
+          <t>National Treasury / World Bank</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -928,7 +932,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -940,7 +944,7 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -959,7 +963,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -995,7 +999,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross, CBK headline figure; composition and encumbrances not stated (IMF International Liquidity shows US$15.361B at Jul-26, gold negligible)</t>
+          <t>CBK gross reserves; gold negligible; swap, forward and short-term liability encumbrances not netted</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1027,7 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>4.632</v>
+        <v>4.63</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1042,7 +1046,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1105,7 +1109,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>147.265</v>
+        <v>147.3</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1124,7 +1128,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1237,7 +1241,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>17-Jul-26</t>
+          <t>23-Jan-26</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1263,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>21-Aug-26</t>
+          <t>22-Aug-25</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1285,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Jul-26</t>
+          <t>27-Jan-26</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1297,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>None; prior EFF/ECF/RSF expired uncompleted Apr-25; successor talks ongoing</t>
+          <t>None (previous EFF/ECF/RSF expired uncompleted Apr-25; new request Mar-25, no staff-level agreement; Article IV mission expected early Dec-26)</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1353,12 @@
       </c>
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n">
-        <v>147.265</v>
+        <v>147.3</v>
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO 2026E, 15-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1403,7 @@
       <c r="D5" s="2" t="n"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO 2026E, 15-Oct-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-23 12:04
</commit_message>
<xml_diff>
--- a/models/sovereigns/Kenya_Sovereign_Model.xlsx
+++ b/models/sovereigns/Kenya_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 15-Oct-26</t>
+          <t>as of 23-Oct-26</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 19-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/kenya.json</t>
+          <t>built 23-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/kenya.json</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CBK MPC press release</t>
+          <t>CBK MPC press release (CBR held, fourth consecutive hold)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>15-Oct-26</t>
+          <t>30-Sep-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>4.5</v>
+        <v>4.9</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -726,19 +726,15 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>2026F</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
+          <t>S&amp;P forecast as reported in press (tier 3, undated)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -779,17 +775,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>National Treasury and Economic Planning</t>
+          <t>National Treasury</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Jun-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Public debt Ksh13.01tn; National Treasury anchor 55% of GDP</t>
+          <t>Public debt Ksh13.01tn; anchor 55% of GDP</t>
         </is>
       </c>
     </row>
@@ -826,17 +822,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FY2025/26 (projection, Ksh1.199tn deficit)</t>
+          <t>FY2025/26 (projection, Ksh1.199tn deficit; no audited outturn)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>National Treasury and Economic Planning</t>
+          <t>National Treasury</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>15-Oct-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -874,7 +870,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FY2025/26 (approximate, ordinary revenue)</t>
+          <t>FY2025/26 (approximate, share of ordinary revenue)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -884,7 +880,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15-Oct-26</t>
+          <t>Jul-26</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -932,7 +928,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>15-Oct-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -963,7 +959,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>15-Oct-26</t>
+          <t>31-Dec-25</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -999,7 +995,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>CBK gross reserves; gold negligible; swap, forward and short-term liability encumbrances not netted</t>
+          <t>CBK headline gross reserves; gold negligible (IMF International Liquidity). IMF series shows 15.361 for Jul-26; the gap is unexplained</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1042,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>15-Oct-26</t>
+          <t>31-Dec-25</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1128,7 +1124,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>15-Oct-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1297,7 +1293,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>None (previous EFF/ECF/RSF expired uncompleted Apr-25; new request Mar-25, no staff-level agreement; Article IV mission expected early Dec-26)</t>
+          <t>None; previous EFF/ECF/RSF expired uncompleted in Apr-25; new programme requested Mar-25, no staff-level agreement; Article IV mission expected early Dec-26</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1354,7 @@
       <c r="D2" s="2" t="n"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>IMF WEO 2026E, 15-Oct-26</t>
+          <t>IMF WEO, Sep-26</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1399,7 @@
       <c r="D5" s="2" t="n"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>IMF WEO 2026E, 15-Oct-26</t>
+          <t>IMF WEO, Sep-26</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1418,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>National Treasury, FY2025/26 projected (Jul-26 to Jun-26 year), Jul-26</t>
+          <t>National Treasury, FY2025/26 projection (year to Jun-26), Jul-26</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1448,7 @@
       <c r="D8" s="2" t="n"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>National Treasury, Jun-26</t>
+          <t>National Treasury, Jun-26 (FY end)</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1504,7 @@
       <c r="D12" s="2" t="n"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>National Treasury / World Bank, Jun-26; approx., share of ordinary revenue, FY2025/26</t>
+          <t>National Treasury / World Bank, approximate, FY2025/26, Jul-26</t>
         </is>
       </c>
     </row>

</xml_diff>